<commit_message>
filled out excel with pin mappings using gemini (pls validate if possible)
</commit_message>
<xml_diff>
--- a/ProjectPinAssignments.xlsx
+++ b/ProjectPinAssignments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ryangelston/Desktop/sp26/ece362/project/362_smart_knob/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ECE264\362_smart_knob\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B220982E-30D3-CC45-957F-E424DDE5F23B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{853EE482-C7E8-4F7D-A86D-3BB37CAC8C3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20560" yWindow="780" windowWidth="20560" windowHeight="24120" xr2:uid="{D0364854-C5F2-6A4F-A138-C6EDFF05F4AB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D0364854-C5F2-6A4F-A138-C6EDFF05F4AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="107">
   <si>
     <t>Name</t>
   </si>
@@ -231,6 +231,132 @@
   </si>
   <si>
     <t>ADC</t>
+  </si>
+  <si>
+    <t>PWM 0A</t>
+  </si>
+  <si>
+    <t>PWM 0B</t>
+  </si>
+  <si>
+    <t>PWM 1A</t>
+  </si>
+  <si>
+    <t>PWM 1B</t>
+  </si>
+  <si>
+    <t>PWM 2A</t>
+  </si>
+  <si>
+    <t>PWM 2B</t>
+  </si>
+  <si>
+    <t>GPIO 0</t>
+  </si>
+  <si>
+    <t>GPIO 1</t>
+  </si>
+  <si>
+    <t>GPIO 2</t>
+  </si>
+  <si>
+    <t>GPIO 3</t>
+  </si>
+  <si>
+    <t>GPIO 4</t>
+  </si>
+  <si>
+    <t>GPIO 5</t>
+  </si>
+  <si>
+    <t>SIO (Digital In) (used for interrupt</t>
+  </si>
+  <si>
+    <t>GPIO 6</t>
+  </si>
+  <si>
+    <t>SPI CS (Encoder) SIO (Digital Out)</t>
+  </si>
+  <si>
+    <t>SPI0 SCK</t>
+  </si>
+  <si>
+    <t>SPIO RX</t>
+  </si>
+  <si>
+    <t>HX711 Clock (PIO / SIO Bitbanged)</t>
+  </si>
+  <si>
+    <t>HX711 Data (PIO / SIO Bitbanged)</t>
+  </si>
+  <si>
+    <t>GPIO 22</t>
+  </si>
+  <si>
+    <t>GPIO 23</t>
+  </si>
+  <si>
+    <t>Display Clock SPI1 SCK</t>
+  </si>
+  <si>
+    <t>GPIO 10</t>
+  </si>
+  <si>
+    <t>Display Reset (SIO Digital IO)</t>
+  </si>
+  <si>
+    <t>SPI1 TX</t>
+  </si>
+  <si>
+    <t>Chip Select(SIO Digital IO)</t>
+  </si>
+  <si>
+    <t>Data/Command (SIO Digital IO)</t>
+  </si>
+  <si>
+    <t>GPIO 11</t>
+  </si>
+  <si>
+    <t>GPIO 12</t>
+  </si>
+  <si>
+    <t>GPIO 13</t>
+  </si>
+  <si>
+    <t>GPIO 14</t>
+  </si>
+  <si>
+    <t>GPIO 15</t>
+  </si>
+  <si>
+    <t>PWM 7B</t>
+  </si>
+  <si>
+    <t>GPIO 45</t>
+  </si>
+  <si>
+    <t>GPIO 42</t>
+  </si>
+  <si>
+    <t>GPIO 44</t>
+  </si>
+  <si>
+    <t>GPIO 8</t>
+  </si>
+  <si>
+    <t>GPIO 9</t>
+  </si>
+  <si>
+    <t>I2C0 SDA</t>
+  </si>
+  <si>
+    <t>I2C0 SCL</t>
+  </si>
+  <si>
+    <t>PIO (LED has it's own async thing???)</t>
+  </si>
+  <si>
+    <t>GPIO 43</t>
   </si>
 </sst>
 </file>
@@ -703,17 +829,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84824A13-219E-6A40-A98F-D95A60BA928F}">
   <dimension ref="B2:L25"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="3.1640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="32.83203125" style="4" customWidth="1"/>
-    <col min="7" max="7" width="41.1640625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="3.19921875" style="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.796875" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="32.796875" style="4" customWidth="1"/>
+    <col min="7" max="7" width="41.19921875" style="4" customWidth="1"/>
     <col min="8" max="8" width="13.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:12" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:12" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B2" s="12"/>
       <c r="C2" s="13" t="s">
         <v>0</v>
@@ -734,7 +860,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="2:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B3" s="12">
         <v>1</v>
       </c>
@@ -748,10 +874,14 @@
         <v>48</v>
       </c>
       <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="1"/>
-    </row>
-    <row r="4" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="G3" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B4" s="12">
         <v>2</v>
       </c>
@@ -765,10 +895,14 @@
         <v>49</v>
       </c>
       <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="1"/>
-    </row>
-    <row r="5" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="G4" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="5" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B5" s="12">
         <v>3</v>
       </c>
@@ -782,10 +916,14 @@
         <v>50</v>
       </c>
       <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="1"/>
-    </row>
-    <row r="6" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="G5" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="6" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B6" s="12">
         <v>4</v>
       </c>
@@ -799,10 +937,14 @@
         <v>51</v>
       </c>
       <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="1"/>
-    </row>
-    <row r="7" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="G6" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B7" s="12">
         <v>5</v>
       </c>
@@ -816,10 +958,14 @@
         <v>52</v>
       </c>
       <c r="F7" s="5"/>
-      <c r="G7" s="5"/>
-      <c r="H7" s="1"/>
-    </row>
-    <row r="8" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="G7" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B8" s="12">
         <v>6</v>
       </c>
@@ -833,13 +979,17 @@
         <v>53</v>
       </c>
       <c r="F8" s="5"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="1"/>
+      <c r="G8" s="5" t="s">
+        <v>68</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>74</v>
+      </c>
       <c r="L8" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="2:12" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B9" s="12">
         <v>7</v>
       </c>
@@ -853,10 +1003,14 @@
         <v>54</v>
       </c>
       <c r="F9" s="5"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="1"/>
-    </row>
-    <row r="10" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="G9" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="10" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B10" s="12">
         <v>8</v>
       </c>
@@ -870,10 +1024,14 @@
         <v>55</v>
       </c>
       <c r="F10" s="5"/>
-      <c r="G10" s="5"/>
-      <c r="H10" s="1"/>
-    </row>
-    <row r="11" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="G10" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B11" s="12">
         <v>9</v>
       </c>
@@ -885,10 +1043,14 @@
       </c>
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
-      <c r="G11" s="5"/>
-      <c r="H11" s="1"/>
-    </row>
-    <row r="12" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="G11" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B12" s="12">
         <v>10</v>
       </c>
@@ -900,10 +1062,14 @@
       </c>
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
-      <c r="G12" s="5"/>
-      <c r="H12" s="1"/>
-    </row>
-    <row r="13" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="G12" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="13" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B13" s="12">
         <v>11</v>
       </c>
@@ -915,10 +1081,14 @@
       </c>
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
-      <c r="G13" s="5"/>
-      <c r="H13" s="1"/>
-    </row>
-    <row r="14" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="G13" s="5" t="s">
+        <v>83</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B14" s="12">
         <v>12</v>
       </c>
@@ -932,10 +1102,14 @@
         <v>64</v>
       </c>
       <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="1"/>
-    </row>
-    <row r="15" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="G14" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="15" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B15" s="12">
         <v>13</v>
       </c>
@@ -949,10 +1123,14 @@
         <v>64</v>
       </c>
       <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="1"/>
-    </row>
-    <row r="16" spans="2:12" x14ac:dyDescent="0.2">
+      <c r="G15" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="16" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B16" s="12">
         <v>14</v>
       </c>
@@ -964,10 +1142,14 @@
       </c>
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
-      <c r="G16" s="5"/>
-      <c r="H16" s="1"/>
-    </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="G16" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B17" s="12">
         <v>15</v>
       </c>
@@ -981,10 +1163,14 @@
         <v>57</v>
       </c>
       <c r="F17" s="5"/>
-      <c r="G17" s="5"/>
-      <c r="H17" s="1"/>
-    </row>
-    <row r="18" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="G17" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B18" s="12">
         <v>16</v>
       </c>
@@ -998,10 +1184,14 @@
         <v>58</v>
       </c>
       <c r="F18" s="5"/>
-      <c r="G18" s="5"/>
-      <c r="H18" s="1"/>
-    </row>
-    <row r="19" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="G18" s="5" t="s">
+        <v>88</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B19" s="12">
         <v>17</v>
       </c>
@@ -1015,10 +1205,14 @@
         <v>59</v>
       </c>
       <c r="F19" s="5"/>
-      <c r="G19" s="5"/>
-      <c r="H19" s="1"/>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="G19" s="5" t="s">
+        <v>86</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B20" s="12">
         <v>18</v>
       </c>
@@ -1032,10 +1226,14 @@
         <v>60</v>
       </c>
       <c r="F20" s="5"/>
-      <c r="G20" s="5"/>
-      <c r="H20" s="1"/>
-    </row>
-    <row r="21" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="G20" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B21" s="12">
         <v>19</v>
       </c>
@@ -1049,10 +1247,14 @@
         <v>61</v>
       </c>
       <c r="F21" s="5"/>
-      <c r="G21" s="5"/>
-      <c r="H21" s="1"/>
-    </row>
-    <row r="22" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="G21" s="5" t="s">
+        <v>97</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B22" s="12">
         <v>20</v>
       </c>
@@ -1066,10 +1268,14 @@
         <v>62</v>
       </c>
       <c r="F22" s="5"/>
-      <c r="G22" s="5"/>
-      <c r="H22" s="1"/>
-    </row>
-    <row r="23" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="G22" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B23" s="12">
         <v>21</v>
       </c>
@@ -1083,10 +1289,14 @@
         <v>63</v>
       </c>
       <c r="F23" s="5"/>
-      <c r="G23" s="5"/>
-      <c r="H23" s="1"/>
-    </row>
-    <row r="24" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="G23" s="5" t="s">
+        <v>91</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B24" s="12">
         <v>22</v>
       </c>
@@ -1097,7 +1307,7 @@
       <c r="G24" s="5"/>
       <c r="H24" s="1"/>
     </row>
-    <row r="25" spans="2:8" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B25" s="12">
         <v>23</v>
       </c>

</xml_diff>

<commit_message>
changed GPIO for UL/UH to accomodate debugger TX and RX
</commit_message>
<xml_diff>
--- a/ProjectPinAssignments.xlsx
+++ b/ProjectPinAssignments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ECE264\362_smart_knob\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{853EE482-C7E8-4F7D-A86D-3BB37CAC8C3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E540CDF-9C47-4F5A-9037-E10012B51069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D0364854-C5F2-6A4F-A138-C6EDFF05F4AB}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="113">
   <si>
     <t>Name</t>
   </si>
@@ -357,6 +357,24 @@
   </si>
   <si>
     <t>GPIO 43</t>
+  </si>
+  <si>
+    <t>GPIO 16</t>
+  </si>
+  <si>
+    <t>GPIO 17</t>
+  </si>
+  <si>
+    <t>Debugger TX</t>
+  </si>
+  <si>
+    <t>Debugger RX</t>
+  </si>
+  <si>
+    <t>UART0 TX</t>
+  </si>
+  <si>
+    <t>UART0 RX</t>
   </si>
 </sst>
 </file>
@@ -941,7 +959,7 @@
         <v>65</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>71</v>
+        <v>107</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.3">
@@ -962,7 +980,7 @@
         <v>66</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>72</v>
+        <v>108</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.3">
@@ -1300,23 +1318,35 @@
       <c r="B24" s="12">
         <v>22</v>
       </c>
-      <c r="C24" s="5"/>
+      <c r="C24" s="5" t="s">
+        <v>109</v>
+      </c>
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
       <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="1"/>
+      <c r="G24" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="25" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B25" s="12">
         <v>23</v>
       </c>
-      <c r="C25" s="5"/>
+      <c r="C25" s="5" t="s">
+        <v>110</v>
+      </c>
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
       <c r="F25" s="5"/>
-      <c r="G25" s="5"/>
-      <c r="H25" s="1"/>
+      <c r="G25" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>71</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added RP 2350 pin table
</commit_message>
<xml_diff>
--- a/ProjectPinAssignments.xlsx
+++ b/ProjectPinAssignments.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ECE264\362_smart_knob\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E540CDF-9C47-4F5A-9037-E10012B51069}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64ECD31E-E6FF-4A08-A7EC-E4D473972AAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D0364854-C5F2-6A4F-A138-C6EDFF05F4AB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="1" xr2:uid="{D0364854-C5F2-6A4F-A138-C6EDFF05F4AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="RP 2350 Pins" sheetId="6" r:id="rId2"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="850" uniqueCount="282">
   <si>
     <t>Name</t>
   </si>
@@ -269,9 +270,6 @@
     <t>GPIO 5</t>
   </si>
   <si>
-    <t>SIO (Digital In) (used for interrupt</t>
-  </si>
-  <si>
     <t>GPIO 6</t>
   </si>
   <si>
@@ -365,23 +363,533 @@
     <t>GPIO 17</t>
   </si>
   <si>
-    <t>Debugger TX</t>
-  </si>
-  <si>
-    <t>Debugger RX</t>
-  </si>
-  <si>
     <t>UART0 TX</t>
   </si>
   <si>
     <t>UART0 RX</t>
+  </si>
+  <si>
+    <t>SIO (Digital In) (used for interrupt)</t>
+  </si>
+  <si>
+    <t>DEBUG_TX</t>
+  </si>
+  <si>
+    <t>DEBUG_RX</t>
+  </si>
+  <si>
+    <t>USB_SERIAL_RXI</t>
+  </si>
+  <si>
+    <t>USB_SERIAL_TXO</t>
+  </si>
+  <si>
+    <t>TXD</t>
+  </si>
+  <si>
+    <t>RXD</t>
+  </si>
+  <si>
+    <t>UART1 TX</t>
+  </si>
+  <si>
+    <t>UART1 RX</t>
+  </si>
+  <si>
+    <t>GPIO</t>
+  </si>
+  <si>
+    <t>TMC_UH</t>
+  </si>
+  <si>
+    <t>SPI1 SCK</t>
+  </si>
+  <si>
+    <t>SPI0 RX</t>
+  </si>
+  <si>
+    <t>SIO</t>
+  </si>
+  <si>
+    <t>PIO0_0</t>
+  </si>
+  <si>
+    <t>PIO1_0</t>
+  </si>
+  <si>
+    <t>PIO2_0</t>
+  </si>
+  <si>
+    <t>GPCK0</t>
+  </si>
+  <si>
+    <t>SPI0 CSn</t>
+  </si>
+  <si>
+    <t>PIO0_1</t>
+  </si>
+  <si>
+    <t>PIO1_1</t>
+  </si>
+  <si>
+    <t>PIO2_1</t>
+  </si>
+  <si>
+    <t>GPCK1</t>
+  </si>
+  <si>
+    <t>UART0 CTS</t>
+  </si>
+  <si>
+    <t>I2C1 SDA</t>
+  </si>
+  <si>
+    <t>PIO0_2</t>
+  </si>
+  <si>
+    <t>PIO1_2</t>
+  </si>
+  <si>
+    <t>PIO2_2</t>
+  </si>
+  <si>
+    <t>SPI0 TX</t>
+  </si>
+  <si>
+    <t>UART0 RTS</t>
+  </si>
+  <si>
+    <t>I2C1 SCL</t>
+  </si>
+  <si>
+    <t>PIO0_3</t>
+  </si>
+  <si>
+    <t>PIO1_3</t>
+  </si>
+  <si>
+    <t>PIO2_3</t>
+  </si>
+  <si>
+    <t>PIO0_4</t>
+  </si>
+  <si>
+    <t>PIO1_4</t>
+  </si>
+  <si>
+    <t>PIO2_4</t>
+  </si>
+  <si>
+    <t>GPCK2</t>
+  </si>
+  <si>
+    <t>PIO0_5</t>
+  </si>
+  <si>
+    <t>PIO1_5</t>
+  </si>
+  <si>
+    <t>PIO2_5</t>
+  </si>
+  <si>
+    <t>GPCK3</t>
+  </si>
+  <si>
+    <t>UART1 CTS</t>
+  </si>
+  <si>
+    <t>PWM 3A</t>
+  </si>
+  <si>
+    <t>PIO0_6</t>
+  </si>
+  <si>
+    <t>PIO1_6</t>
+  </si>
+  <si>
+    <t>PIO2_6</t>
+  </si>
+  <si>
+    <t>UART1 RTS</t>
+  </si>
+  <si>
+    <t>PWM 3B</t>
+  </si>
+  <si>
+    <t>PIO0_7</t>
+  </si>
+  <si>
+    <t>PIO1_7</t>
+  </si>
+  <si>
+    <t>PIO2_7</t>
+  </si>
+  <si>
+    <t>SPI1 RX</t>
+  </si>
+  <si>
+    <t>PWM 4A</t>
+  </si>
+  <si>
+    <t>PIO0_8</t>
+  </si>
+  <si>
+    <t>PIO1_8</t>
+  </si>
+  <si>
+    <t>PIO2_8</t>
+  </si>
+  <si>
+    <t>SPI1 CSn</t>
+  </si>
+  <si>
+    <t>PWM 4B</t>
+  </si>
+  <si>
+    <t>PIO0_9</t>
+  </si>
+  <si>
+    <t>PIO1_9</t>
+  </si>
+  <si>
+    <t>PIO2_9</t>
+  </si>
+  <si>
+    <t>PWM 5A</t>
+  </si>
+  <si>
+    <t>PIO0_10</t>
+  </si>
+  <si>
+    <t>PIO1_10</t>
+  </si>
+  <si>
+    <t>PIO2_10</t>
+  </si>
+  <si>
+    <t>PWM 5B</t>
+  </si>
+  <si>
+    <t>PIO0_11</t>
+  </si>
+  <si>
+    <t>PIO1_11</t>
+  </si>
+  <si>
+    <t>PIO2_11</t>
+  </si>
+  <si>
+    <t>PWM 6A</t>
+  </si>
+  <si>
+    <t>PIO0_12</t>
+  </si>
+  <si>
+    <t>PIO1_12</t>
+  </si>
+  <si>
+    <t>PIO2_12</t>
+  </si>
+  <si>
+    <t>PWM 6B</t>
+  </si>
+  <si>
+    <t>PIO0_13</t>
+  </si>
+  <si>
+    <t>PIO1_13</t>
+  </si>
+  <si>
+    <t>PIO2_13</t>
+  </si>
+  <si>
+    <t>PWM 7A</t>
+  </si>
+  <si>
+    <t>PIO0_14</t>
+  </si>
+  <si>
+    <t>PIO1_14</t>
+  </si>
+  <si>
+    <t>PIO2_14</t>
+  </si>
+  <si>
+    <t>PIO0_15</t>
+  </si>
+  <si>
+    <t>PIO1_15</t>
+  </si>
+  <si>
+    <t>PIO2_15</t>
+  </si>
+  <si>
+    <t>PIO0_16</t>
+  </si>
+  <si>
+    <t>PIO1_16</t>
+  </si>
+  <si>
+    <t>PIO2_16</t>
+  </si>
+  <si>
+    <t>PIO0_17</t>
+  </si>
+  <si>
+    <t>PIO1_17</t>
+  </si>
+  <si>
+    <t>PIO2_17</t>
+  </si>
+  <si>
+    <t>PIO0_18</t>
+  </si>
+  <si>
+    <t>PIO1_18</t>
+  </si>
+  <si>
+    <t>PIO2_18</t>
+  </si>
+  <si>
+    <t>PIO0_19</t>
+  </si>
+  <si>
+    <t>PIO1_19</t>
+  </si>
+  <si>
+    <t>PIO2_19</t>
+  </si>
+  <si>
+    <t>PIO0_20</t>
+  </si>
+  <si>
+    <t>PIO1_20</t>
+  </si>
+  <si>
+    <t>PIO2_20</t>
+  </si>
+  <si>
+    <t>PIO0_21</t>
+  </si>
+  <si>
+    <t>PIO1_21</t>
+  </si>
+  <si>
+    <t>PIO2_21</t>
+  </si>
+  <si>
+    <t>PIO0_22</t>
+  </si>
+  <si>
+    <t>PIO1_22</t>
+  </si>
+  <si>
+    <t>PIO2_22</t>
+  </si>
+  <si>
+    <t>PIO0_23</t>
+  </si>
+  <si>
+    <t>PIO1_23</t>
+  </si>
+  <si>
+    <t>PIO2_23</t>
+  </si>
+  <si>
+    <t>PIO0_24</t>
+  </si>
+  <si>
+    <t>PIO1_24</t>
+  </si>
+  <si>
+    <t>PIO2_24</t>
+  </si>
+  <si>
+    <t>PIO0_25</t>
+  </si>
+  <si>
+    <t>PIO1_25</t>
+  </si>
+  <si>
+    <t>PIO2_25</t>
+  </si>
+  <si>
+    <t>PIO0_26</t>
+  </si>
+  <si>
+    <t>PIO1_26</t>
+  </si>
+  <si>
+    <t>PIO2_26</t>
+  </si>
+  <si>
+    <t>PIO0_27</t>
+  </si>
+  <si>
+    <t>PIO1_27</t>
+  </si>
+  <si>
+    <t>PIO2_27</t>
+  </si>
+  <si>
+    <t>PIO0_28</t>
+  </si>
+  <si>
+    <t>PIO1_28</t>
+  </si>
+  <si>
+    <t>PIO2_28</t>
+  </si>
+  <si>
+    <t>PIO0_29</t>
+  </si>
+  <si>
+    <t>PIO1_29</t>
+  </si>
+  <si>
+    <t>PIO2_29</t>
+  </si>
+  <si>
+    <t>PIO0_30</t>
+  </si>
+  <si>
+    <t>PIO1_30</t>
+  </si>
+  <si>
+    <t>PIO2_30</t>
+  </si>
+  <si>
+    <t>PIO0_31</t>
+  </si>
+  <si>
+    <t>PIO1_31</t>
+  </si>
+  <si>
+    <t>PIO2_31</t>
+  </si>
+  <si>
+    <t>PWM 8A</t>
+  </si>
+  <si>
+    <t>PWM 8B</t>
+  </si>
+  <si>
+    <t>PWM 9A</t>
+  </si>
+  <si>
+    <t>PWM 9B</t>
+  </si>
+  <si>
+    <t>PWM 10A</t>
+  </si>
+  <si>
+    <t>PWM 10B</t>
+  </si>
+  <si>
+    <t>PWM 11A</t>
+  </si>
+  <si>
+    <t>PWM 11B</t>
+  </si>
+  <si>
+    <t>ADC 0</t>
+  </si>
+  <si>
+    <t>ADC 1</t>
+  </si>
+  <si>
+    <t>ADC 2</t>
+  </si>
+  <si>
+    <t>ADC 3</t>
+  </si>
+  <si>
+    <t>ADC 4</t>
+  </si>
+  <si>
+    <t>ADC 5</t>
+  </si>
+  <si>
+    <t>ADC 6</t>
+  </si>
+  <si>
+    <t>ADC 7</t>
+  </si>
+  <si>
+    <t>F0</t>
+  </si>
+  <si>
+    <t>F1</t>
+  </si>
+  <si>
+    <t>F2</t>
+  </si>
+  <si>
+    <t>F3</t>
+  </si>
+  <si>
+    <t>F4</t>
+  </si>
+  <si>
+    <t>F5</t>
+  </si>
+  <si>
+    <t>F6</t>
+  </si>
+  <si>
+    <t>F7</t>
+  </si>
+  <si>
+    <t>F8</t>
+  </si>
+  <si>
+    <t>F9</t>
+  </si>
+  <si>
+    <t>F10</t>
+  </si>
+  <si>
+    <t>F11</t>
+  </si>
+  <si>
+    <t>F12</t>
+  </si>
+  <si>
+    <t>USB OVR</t>
+  </si>
+  <si>
+    <t>PROC0</t>
+  </si>
+  <si>
+    <t>USB VBUS</t>
+  </si>
+  <si>
+    <t>PROC1</t>
+  </si>
+  <si>
+    <t>HSTX</t>
+  </si>
+  <si>
+    <t>Usage</t>
+  </si>
+  <si>
+    <t>Target Fcn</t>
+  </si>
+  <si>
+    <t>(Avail)</t>
+  </si>
+  <si>
+    <t>Proton Button</t>
+  </si>
+  <si>
+    <t>Proton LED</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -396,8 +904,14 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -446,8 +960,20 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBE2D5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -470,11 +996,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -512,12 +1053,36 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <colors>
+    <mruColors>
+      <color rgb="FFFBE2D5"/>
+      <color rgb="FFDE7272"/>
+    </mruColors>
+  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -846,7 +1411,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84824A13-219E-6A40-A98F-D95A60BA928F}">
-  <dimension ref="B2:L25"/>
+  <dimension ref="B2:L27"/>
   <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="3.19921875" style="3" bestFit="1" customWidth="1"/>
@@ -893,10 +1458,10 @@
       </c>
       <c r="F3" s="5"/>
       <c r="G3" s="5" t="s">
+        <v>110</v>
+      </c>
+      <c r="H3" s="1" t="s">
         <v>77</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="4" spans="2:12" x14ac:dyDescent="0.3">
@@ -959,7 +1524,7 @@
         <v>65</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7" spans="2:12" x14ac:dyDescent="0.3">
@@ -980,7 +1545,7 @@
         <v>66</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" spans="2:12" x14ac:dyDescent="0.3">
@@ -1022,10 +1587,10 @@
       </c>
       <c r="F9" s="5"/>
       <c r="G9" s="5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="2:12" x14ac:dyDescent="0.3">
@@ -1062,10 +1627,10 @@
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
       <c r="G11" s="5" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="12" spans="2:12" x14ac:dyDescent="0.3">
@@ -1081,10 +1646,10 @@
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
       <c r="G12" s="5" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="13" spans="2:12" x14ac:dyDescent="0.3">
@@ -1100,10 +1665,10 @@
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
       <c r="G13" s="5" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="14" spans="2:12" x14ac:dyDescent="0.3">
@@ -1121,10 +1686,10 @@
       </c>
       <c r="F14" s="5"/>
       <c r="G14" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="H14" s="1" t="s">
         <v>105</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="15" spans="2:12" x14ac:dyDescent="0.3">
@@ -1142,10 +1707,10 @@
       </c>
       <c r="F15" s="5"/>
       <c r="G15" s="5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="16" spans="2:12" x14ac:dyDescent="0.3">
@@ -1161,10 +1726,10 @@
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
       <c r="G16" s="5" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" spans="2:8" x14ac:dyDescent="0.3">
@@ -1182,10 +1747,10 @@
       </c>
       <c r="F17" s="5"/>
       <c r="G17" s="5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.3">
@@ -1203,10 +1768,10 @@
       </c>
       <c r="F18" s="5"/>
       <c r="G18" s="5" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" spans="2:8" x14ac:dyDescent="0.3">
@@ -1224,10 +1789,10 @@
       </c>
       <c r="F19" s="5"/>
       <c r="G19" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="H19" s="1" t="s">
         <v>86</v>
-      </c>
-      <c r="H19" s="1" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.3">
@@ -1245,10 +1810,10 @@
       </c>
       <c r="F20" s="5"/>
       <c r="G20" s="5" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="H20" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="21" spans="2:8" x14ac:dyDescent="0.3">
@@ -1266,10 +1831,10 @@
       </c>
       <c r="F21" s="5"/>
       <c r="G21" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="H21" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="22" spans="2:8" x14ac:dyDescent="0.3">
@@ -1287,10 +1852,10 @@
       </c>
       <c r="F22" s="5"/>
       <c r="G22" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="H22" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="23" spans="2:8" x14ac:dyDescent="0.3">
@@ -1308,10 +1873,10 @@
       </c>
       <c r="F23" s="5"/>
       <c r="G23" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H23" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="24" spans="2:8" x14ac:dyDescent="0.3">
@@ -1319,13 +1884,13 @@
         <v>22</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
       <c r="F24" s="5"/>
       <c r="G24" s="5" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="H24" s="1" t="s">
         <v>72</v>
@@ -1336,16 +1901,2501 @@
         <v>23</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
       <c r="F25" s="5"/>
       <c r="G25" s="5" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="H25" s="1" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B26" s="12">
+        <v>24</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>113</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="H26" s="1"/>
+    </row>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B27" s="12">
+        <v>25</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="H27" s="1"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3AA3AC0-7217-4DB3-9834-2C3B6854440A}">
+  <dimension ref="A1:P49"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="13.796875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="15" t="s">
+        <v>119</v>
+      </c>
+      <c r="B1" s="15" t="s">
+        <v>277</v>
+      </c>
+      <c r="C1" s="15" t="s">
+        <v>278</v>
+      </c>
+      <c r="D1" s="15" t="s">
+        <v>259</v>
+      </c>
+      <c r="E1" s="15" t="s">
+        <v>260</v>
+      </c>
+      <c r="F1" s="15" t="s">
+        <v>261</v>
+      </c>
+      <c r="G1" s="15" t="s">
+        <v>262</v>
+      </c>
+      <c r="H1" s="15" t="s">
+        <v>263</v>
+      </c>
+      <c r="I1" s="15" t="s">
+        <v>264</v>
+      </c>
+      <c r="J1" s="15" t="s">
+        <v>265</v>
+      </c>
+      <c r="K1" s="15" t="s">
+        <v>266</v>
+      </c>
+      <c r="L1" s="15" t="s">
+        <v>267</v>
+      </c>
+      <c r="M1" s="15" t="s">
+        <v>268</v>
+      </c>
+      <c r="N1" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="O1" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="P1" s="15" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="16">
+        <v>0</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="E2" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="F2" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="G2" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="H2" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I2" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="J2" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="K2" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="L2" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M2" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="N2" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O2" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P2" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="16">
+        <v>1</v>
+      </c>
+      <c r="B3" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C3" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D3" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="E3" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="F3" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="G3" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="H3" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I3" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="J3" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="K3" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="L3" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M3" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="N3" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O3" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P3" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="16">
+        <v>2</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="E4" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="F4" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="G4" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="H4" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I4" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="J4" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="K4" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="L4" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M4" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N4" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O4" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P4" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="16">
+        <v>3</v>
+      </c>
+      <c r="B5" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="C5" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="D5" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="E5" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="F5" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="G5" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="H5" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I5" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="J5" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="K5" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="L5" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M5" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N5" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O5" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P5" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="16">
+        <v>4</v>
+      </c>
+      <c r="B6" s="20" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="F6" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="G6" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I6" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="J6" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="K6" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="L6" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M6" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="N6" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O6" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P6" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="16">
+        <v>5</v>
+      </c>
+      <c r="B7" s="20" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F7" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="G7" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="H7" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I7" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="J7" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="K7" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="L7" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M7" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="N7" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O7" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P7" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="16">
+        <v>6</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="D8" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="F8" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="G8" s="20" t="s">
+        <v>153</v>
+      </c>
+      <c r="H8" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="I8" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="J8" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="K8" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="L8" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M8" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N8" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O8" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P8" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="16">
+        <v>7</v>
+      </c>
+      <c r="B9" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="F9" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="G9" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="H9" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I9" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="J9" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="K9" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="L9" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M9" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N9" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O9" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P9" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="16">
+        <v>8</v>
+      </c>
+      <c r="B10" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="E10" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="F10" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="G10" s="19" t="s">
+        <v>163</v>
+      </c>
+      <c r="H10" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I10" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="J10" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="K10" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="L10" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M10" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="N10" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O10" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P10" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="16">
+        <v>9</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="E11" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F11" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="G11" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="H11" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I11" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="J11" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="K11" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="L11" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M11" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="N11" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O11" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P11" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="16">
+        <v>10</v>
+      </c>
+      <c r="B12" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="G12" s="15" t="s">
+        <v>172</v>
+      </c>
+      <c r="H12" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I12" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="J12" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="K12" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="L12" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M12" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N12" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O12" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P12" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="16">
+        <v>11</v>
+      </c>
+      <c r="B13" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C13" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="E13" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="F13" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="G13" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="H13" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I13" s="15" t="s">
+        <v>177</v>
+      </c>
+      <c r="J13" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="K13" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="L13" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M13" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N13" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O13" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P13" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="16">
+        <v>12</v>
+      </c>
+      <c r="B14" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="E14" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="F14" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="H14" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I14" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="J14" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="K14" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="L14" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M14" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="N14" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O14" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P14" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="16">
+        <v>13</v>
+      </c>
+      <c r="B15" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C15" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="E15" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="F15" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="G15" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="H15" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I15" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="J15" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="K15" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="L15" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M15" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="N15" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O15" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P15" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="16">
+        <v>14</v>
+      </c>
+      <c r="B16" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="E16" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="F16" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="G16" s="15" t="s">
+        <v>188</v>
+      </c>
+      <c r="H16" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I16" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="J16" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="K16" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="L16" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M16" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N16" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O16" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P16" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="17" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="16">
+        <v>15</v>
+      </c>
+      <c r="B17" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C17" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="E17" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="F17" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="G17" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="H17" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I17" s="15" t="s">
+        <v>192</v>
+      </c>
+      <c r="J17" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="K17" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="L17" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M17" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N17" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O17" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P17" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="18" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="16">
+        <v>16</v>
+      </c>
+      <c r="B18" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="E18" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="F18" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="G18" s="15" t="s">
+        <v>65</v>
+      </c>
+      <c r="H18" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I18" s="15" t="s">
+        <v>195</v>
+      </c>
+      <c r="J18" s="15" t="s">
+        <v>196</v>
+      </c>
+      <c r="K18" s="15" t="s">
+        <v>197</v>
+      </c>
+      <c r="L18" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M18" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="N18" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O18" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P18" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="19" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="16">
+        <v>17</v>
+      </c>
+      <c r="B19" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="E19" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="F19" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="G19" s="15" t="s">
+        <v>66</v>
+      </c>
+      <c r="H19" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I19" s="15" t="s">
+        <v>198</v>
+      </c>
+      <c r="J19" s="15" t="s">
+        <v>199</v>
+      </c>
+      <c r="K19" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="L19" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M19" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="N19" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O19" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P19" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="20" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="16">
+        <v>18</v>
+      </c>
+      <c r="B20" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="E20" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="F20" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="G20" s="15" t="s">
+        <v>67</v>
+      </c>
+      <c r="H20" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I20" s="15" t="s">
+        <v>201</v>
+      </c>
+      <c r="J20" s="15" t="s">
+        <v>202</v>
+      </c>
+      <c r="K20" s="15" t="s">
+        <v>203</v>
+      </c>
+      <c r="L20" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M20" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N20" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O20" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P20" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="21" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="16">
+        <v>19</v>
+      </c>
+      <c r="B21" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C21" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="E21" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="F21" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="G21" s="15" t="s">
+        <v>68</v>
+      </c>
+      <c r="H21" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I21" s="15" t="s">
+        <v>204</v>
+      </c>
+      <c r="J21" s="15" t="s">
+        <v>205</v>
+      </c>
+      <c r="K21" s="15" t="s">
+        <v>206</v>
+      </c>
+      <c r="L21" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M21" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N21" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O21" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P21" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="22" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="16">
+        <v>20</v>
+      </c>
+      <c r="B22" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="E22" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="F22" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="G22" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="H22" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I22" s="15" t="s">
+        <v>207</v>
+      </c>
+      <c r="J22" s="15" t="s">
+        <v>208</v>
+      </c>
+      <c r="K22" s="15" t="s">
+        <v>209</v>
+      </c>
+      <c r="L22" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M22" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="N22" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O22" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P22" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="23" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="17">
+        <v>21</v>
+      </c>
+      <c r="B23" s="18" t="s">
+        <v>280</v>
+      </c>
+      <c r="C23" s="18"/>
+      <c r="D23" s="18" t="s">
+        <v>128</v>
+      </c>
+      <c r="E23" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="F23" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="G23" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="H23" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="I23" s="18" t="s">
+        <v>210</v>
+      </c>
+      <c r="J23" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="K23" s="18" t="s">
+        <v>212</v>
+      </c>
+      <c r="L23" s="18" t="s">
+        <v>274</v>
+      </c>
+      <c r="M23" s="18" t="s">
+        <v>151</v>
+      </c>
+      <c r="N23" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="O23" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="P23" s="18" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="24" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="17">
+        <v>22</v>
+      </c>
+      <c r="B24" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C24" s="18"/>
+      <c r="D24" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="E24" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="F24" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="G24" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="H24" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="I24" s="18" t="s">
+        <v>213</v>
+      </c>
+      <c r="J24" s="18" t="s">
+        <v>214</v>
+      </c>
+      <c r="K24" s="18" t="s">
+        <v>215</v>
+      </c>
+      <c r="L24" s="18" t="s">
+        <v>272</v>
+      </c>
+      <c r="M24" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="N24" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="O24" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="P24" s="18" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="25" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="17">
+        <v>23</v>
+      </c>
+      <c r="B25" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18" t="s">
+        <v>138</v>
+      </c>
+      <c r="E25" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="F25" s="18" t="s">
+        <v>140</v>
+      </c>
+      <c r="G25" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="H25" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="I25" s="18" t="s">
+        <v>216</v>
+      </c>
+      <c r="J25" s="18" t="s">
+        <v>217</v>
+      </c>
+      <c r="K25" s="18" t="s">
+        <v>218</v>
+      </c>
+      <c r="L25" s="18" t="s">
+        <v>274</v>
+      </c>
+      <c r="M25" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="N25" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="O25" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="P25" s="18" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="26" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="17">
+        <v>24</v>
+      </c>
+      <c r="B26" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18" t="s">
+        <v>162</v>
+      </c>
+      <c r="E26" s="18" t="s">
+        <v>117</v>
+      </c>
+      <c r="F26" s="18" t="s">
+        <v>102</v>
+      </c>
+      <c r="G26" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="H26" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="I26" s="18" t="s">
+        <v>219</v>
+      </c>
+      <c r="J26" s="18" t="s">
+        <v>220</v>
+      </c>
+      <c r="K26" s="18" t="s">
+        <v>221</v>
+      </c>
+      <c r="L26" s="18" t="s">
+        <v>272</v>
+      </c>
+      <c r="M26" s="18" t="s">
+        <v>127</v>
+      </c>
+      <c r="N26" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="O26" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="P26" s="18" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="27" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="17">
+        <v>25</v>
+      </c>
+      <c r="B27" s="18" t="s">
+        <v>281</v>
+      </c>
+      <c r="C27" s="18"/>
+      <c r="D27" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="E27" s="18" t="s">
+        <v>118</v>
+      </c>
+      <c r="F27" s="18" t="s">
+        <v>103</v>
+      </c>
+      <c r="G27" s="18" t="s">
+        <v>168</v>
+      </c>
+      <c r="H27" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="I27" s="18" t="s">
+        <v>222</v>
+      </c>
+      <c r="J27" s="18" t="s">
+        <v>223</v>
+      </c>
+      <c r="K27" s="18" t="s">
+        <v>224</v>
+      </c>
+      <c r="L27" s="18" t="s">
+        <v>274</v>
+      </c>
+      <c r="M27" s="18" t="s">
+        <v>132</v>
+      </c>
+      <c r="N27" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="O27" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="P27" s="18" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="28" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A28" s="17">
+        <v>26</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>280</v>
+      </c>
+      <c r="C28" s="18"/>
+      <c r="D28" s="18" t="s">
+        <v>121</v>
+      </c>
+      <c r="E28" s="18" t="s">
+        <v>152</v>
+      </c>
+      <c r="F28" s="18" t="s">
+        <v>134</v>
+      </c>
+      <c r="G28" s="18" t="s">
+        <v>172</v>
+      </c>
+      <c r="H28" s="18" t="s">
+        <v>123</v>
+      </c>
+      <c r="I28" s="18" t="s">
+        <v>225</v>
+      </c>
+      <c r="J28" s="18" t="s">
+        <v>226</v>
+      </c>
+      <c r="K28" s="18" t="s">
+        <v>227</v>
+      </c>
+      <c r="L28" s="18" t="s">
+        <v>272</v>
+      </c>
+      <c r="M28" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="N28" s="18" t="s">
+        <v>251</v>
+      </c>
+      <c r="O28" s="18" t="s">
+        <v>59</v>
+      </c>
+      <c r="P28" s="18" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="29" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="16">
+        <v>27</v>
+      </c>
+      <c r="B29" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C29" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="E29" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="F29" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="G29" s="15" t="s">
+        <v>176</v>
+      </c>
+      <c r="H29" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I29" s="15" t="s">
+        <v>228</v>
+      </c>
+      <c r="J29" s="15" t="s">
+        <v>229</v>
+      </c>
+      <c r="K29" s="15" t="s">
+        <v>230</v>
+      </c>
+      <c r="L29" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M29" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N29" s="15" t="s">
+        <v>252</v>
+      </c>
+      <c r="O29" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="P29" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="30" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="16">
+        <v>28</v>
+      </c>
+      <c r="B30" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="E30" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="F30" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="G30" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="H30" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I30" s="15" t="s">
+        <v>231</v>
+      </c>
+      <c r="J30" s="15" t="s">
+        <v>232</v>
+      </c>
+      <c r="K30" s="15" t="s">
+        <v>233</v>
+      </c>
+      <c r="L30" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M30" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="N30" s="15" t="s">
+        <v>253</v>
+      </c>
+      <c r="O30" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P30" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="31" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="16">
+        <v>29</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="E31" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="F31" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="G31" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="H31" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I31" s="15" t="s">
+        <v>234</v>
+      </c>
+      <c r="J31" s="15" t="s">
+        <v>235</v>
+      </c>
+      <c r="K31" s="15" t="s">
+        <v>236</v>
+      </c>
+      <c r="L31" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M31" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="N31" s="15" t="s">
+        <v>254</v>
+      </c>
+      <c r="O31" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P31" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A32" s="16">
+        <v>30</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="E32" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="F32" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="G32" s="15" t="s">
+        <v>188</v>
+      </c>
+      <c r="H32" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I32" s="15" t="s">
+        <v>237</v>
+      </c>
+      <c r="J32" s="15" t="s">
+        <v>238</v>
+      </c>
+      <c r="K32" s="15" t="s">
+        <v>239</v>
+      </c>
+      <c r="L32" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M32" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N32" s="15" t="s">
+        <v>255</v>
+      </c>
+      <c r="O32" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P32" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="33" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="16">
+        <v>31</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="F33" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="G33" s="15" t="s">
+        <v>96</v>
+      </c>
+      <c r="H33" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I33" s="15" t="s">
+        <v>240</v>
+      </c>
+      <c r="J33" s="15" t="s">
+        <v>241</v>
+      </c>
+      <c r="K33" s="15" t="s">
+        <v>242</v>
+      </c>
+      <c r="L33" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M33" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N33" s="15" t="s">
+        <v>256</v>
+      </c>
+      <c r="O33" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P33" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="34" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A34" s="16">
+        <v>32</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="E34" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="F34" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="G34" s="15" t="s">
+        <v>243</v>
+      </c>
+      <c r="H34" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I34" s="15" t="s">
+        <v>124</v>
+      </c>
+      <c r="J34" s="15" t="s">
+        <v>125</v>
+      </c>
+      <c r="K34" s="15" t="s">
+        <v>126</v>
+      </c>
+      <c r="L34" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M34" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="N34" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O34" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P34" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="35" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A35" s="16">
+        <v>33</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="E35" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="F35" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="G35" s="15" t="s">
+        <v>244</v>
+      </c>
+      <c r="H35" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I35" s="15" t="s">
+        <v>129</v>
+      </c>
+      <c r="J35" s="15" t="s">
+        <v>130</v>
+      </c>
+      <c r="K35" s="15" t="s">
+        <v>131</v>
+      </c>
+      <c r="L35" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M35" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="N35" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O35" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P35" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="36" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="16">
+        <v>34</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="E36" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="F36" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="G36" s="15" t="s">
+        <v>245</v>
+      </c>
+      <c r="H36" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I36" s="15" t="s">
+        <v>135</v>
+      </c>
+      <c r="J36" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="K36" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="L36" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M36" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N36" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O36" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P36" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="16">
+        <v>35</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="E37" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="F37" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="G37" s="15" t="s">
+        <v>246</v>
+      </c>
+      <c r="H37" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I37" s="15" t="s">
+        <v>141</v>
+      </c>
+      <c r="J37" s="15" t="s">
+        <v>142</v>
+      </c>
+      <c r="K37" s="15" t="s">
+        <v>143</v>
+      </c>
+      <c r="L37" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M37" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N37" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O37" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P37" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="16">
+        <v>36</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D38" s="15" t="s">
+        <v>122</v>
+      </c>
+      <c r="E38" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="F38" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="G38" s="15" t="s">
+        <v>247</v>
+      </c>
+      <c r="H38" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I38" s="15" t="s">
+        <v>144</v>
+      </c>
+      <c r="J38" s="15" t="s">
+        <v>145</v>
+      </c>
+      <c r="K38" s="15" t="s">
+        <v>146</v>
+      </c>
+      <c r="L38" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M38" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="N38" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O38" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P38" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="16">
+        <v>37</v>
+      </c>
+      <c r="B39" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C39" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D39" s="15" t="s">
+        <v>128</v>
+      </c>
+      <c r="E39" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F39" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="G39" s="15" t="s">
+        <v>248</v>
+      </c>
+      <c r="H39" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I39" s="15" t="s">
+        <v>148</v>
+      </c>
+      <c r="J39" s="15" t="s">
+        <v>149</v>
+      </c>
+      <c r="K39" s="15" t="s">
+        <v>150</v>
+      </c>
+      <c r="L39" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M39" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="N39" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O39" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P39" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A40" s="16">
+        <v>38</v>
+      </c>
+      <c r="B40" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C40" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D40" s="15" t="s">
+        <v>79</v>
+      </c>
+      <c r="E40" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="F40" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="G40" s="15" t="s">
+        <v>249</v>
+      </c>
+      <c r="H40" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I40" s="15" t="s">
+        <v>154</v>
+      </c>
+      <c r="J40" s="15" t="s">
+        <v>155</v>
+      </c>
+      <c r="K40" s="15" t="s">
+        <v>156</v>
+      </c>
+      <c r="L40" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M40" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N40" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O40" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P40" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A41" s="16">
+        <v>39</v>
+      </c>
+      <c r="B41" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C41" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D41" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="E41" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="F41" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="G41" s="15" t="s">
+        <v>250</v>
+      </c>
+      <c r="H41" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I41" s="15" t="s">
+        <v>159</v>
+      </c>
+      <c r="J41" s="15" t="s">
+        <v>160</v>
+      </c>
+      <c r="K41" s="15" t="s">
+        <v>161</v>
+      </c>
+      <c r="L41" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M41" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N41" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="O41" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P41" s="15" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="42" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A42" s="16">
+        <v>40</v>
+      </c>
+      <c r="B42" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C42" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D42" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="E42" s="15" t="s">
+        <v>117</v>
+      </c>
+      <c r="F42" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="G42" s="15" t="s">
+        <v>243</v>
+      </c>
+      <c r="H42" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I42" s="15" t="s">
+        <v>164</v>
+      </c>
+      <c r="J42" s="15" t="s">
+        <v>165</v>
+      </c>
+      <c r="K42" s="15" t="s">
+        <v>166</v>
+      </c>
+      <c r="L42" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M42" s="15" t="s">
+        <v>127</v>
+      </c>
+      <c r="N42" s="15" t="s">
+        <v>251</v>
+      </c>
+      <c r="O42" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P42" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="43" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A43" s="16">
+        <v>41</v>
+      </c>
+      <c r="B43" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C43" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D43" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="E43" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="F43" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="G43" s="15" t="s">
+        <v>244</v>
+      </c>
+      <c r="H43" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I43" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="J43" s="15" t="s">
+        <v>170</v>
+      </c>
+      <c r="K43" s="15" t="s">
+        <v>171</v>
+      </c>
+      <c r="L43" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M43" s="15" t="s">
+        <v>132</v>
+      </c>
+      <c r="N43" s="15" t="s">
+        <v>252</v>
+      </c>
+      <c r="O43" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P43" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="44" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A44" s="16">
+        <v>42</v>
+      </c>
+      <c r="B44" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C44" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D44" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="E44" s="15" t="s">
+        <v>152</v>
+      </c>
+      <c r="F44" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="G44" s="15" t="s">
+        <v>245</v>
+      </c>
+      <c r="H44" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I44" s="15" t="s">
+        <v>173</v>
+      </c>
+      <c r="J44" s="15" t="s">
+        <v>174</v>
+      </c>
+      <c r="K44" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="L44" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M44" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N44" s="15" t="s">
+        <v>253</v>
+      </c>
+      <c r="O44" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P44" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="45" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A45" s="16">
+        <v>43</v>
+      </c>
+      <c r="B45" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C45" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D45" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="E45" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="F45" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="G45" s="15" t="s">
+        <v>246</v>
+      </c>
+      <c r="H45" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I45" s="15" t="s">
+        <v>177</v>
+      </c>
+      <c r="J45" s="15" t="s">
+        <v>178</v>
+      </c>
+      <c r="K45" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="L45" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M45" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N45" s="15" t="s">
+        <v>254</v>
+      </c>
+      <c r="O45" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P45" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="46" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A46" s="16">
+        <v>44</v>
+      </c>
+      <c r="B46" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C46" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D46" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="E46" s="15" t="s">
+        <v>108</v>
+      </c>
+      <c r="F46" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="G46" s="15" t="s">
+        <v>247</v>
+      </c>
+      <c r="H46" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I46" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="J46" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="K46" s="15" t="s">
+        <v>183</v>
+      </c>
+      <c r="L46" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M46" s="15" t="s">
+        <v>147</v>
+      </c>
+      <c r="N46" s="15" t="s">
+        <v>255</v>
+      </c>
+      <c r="O46" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P46" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="47" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A47" s="16">
+        <v>45</v>
+      </c>
+      <c r="B47" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C47" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D47" s="15" t="s">
+        <v>167</v>
+      </c>
+      <c r="E47" s="15" t="s">
+        <v>109</v>
+      </c>
+      <c r="F47" s="15" t="s">
+        <v>103</v>
+      </c>
+      <c r="G47" s="15" t="s">
+        <v>248</v>
+      </c>
+      <c r="H47" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I47" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="J47" s="15" t="s">
+        <v>186</v>
+      </c>
+      <c r="K47" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="L47" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M47" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="N47" s="15" t="s">
+        <v>256</v>
+      </c>
+      <c r="O47" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P47" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="48" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A48" s="16">
+        <v>46</v>
+      </c>
+      <c r="B48" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C48" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D48" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="E48" s="15" t="s">
+        <v>133</v>
+      </c>
+      <c r="F48" s="15" t="s">
+        <v>134</v>
+      </c>
+      <c r="G48" s="15" t="s">
+        <v>249</v>
+      </c>
+      <c r="H48" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I48" s="15" t="s">
+        <v>189</v>
+      </c>
+      <c r="J48" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="K48" s="15" t="s">
+        <v>191</v>
+      </c>
+      <c r="L48" s="15" t="s">
+        <v>272</v>
+      </c>
+      <c r="M48" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N48" s="15" t="s">
+        <v>257</v>
+      </c>
+      <c r="O48" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P48" s="15" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="49" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A49" s="16">
+        <v>47</v>
+      </c>
+      <c r="B49" s="15" t="s">
+        <v>279</v>
+      </c>
+      <c r="C49" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="D49" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="E49" s="15" t="s">
+        <v>139</v>
+      </c>
+      <c r="F49" s="15" t="s">
+        <v>140</v>
+      </c>
+      <c r="G49" s="15" t="s">
+        <v>250</v>
+      </c>
+      <c r="H49" s="15" t="s">
+        <v>123</v>
+      </c>
+      <c r="I49" s="15" t="s">
+        <v>192</v>
+      </c>
+      <c r="J49" s="15" t="s">
+        <v>193</v>
+      </c>
+      <c r="K49" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="L49" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="M49" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="N49" s="15" t="s">
+        <v>258</v>
+      </c>
+      <c r="O49" s="15" t="s">
+        <v>276</v>
+      </c>
+      <c r="P49" s="15" t="s">
+        <v>275</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added LDR pin in excel
</commit_message>
<xml_diff>
--- a/ProjectPinAssignments.xlsx
+++ b/ProjectPinAssignments.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ECE264\362_smart_knob\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A52BF67C-8CAE-4446-97E0-817E6E428493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22CC351A-8DAB-49D0-9EBC-DFE290766685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{D0364854-C5F2-6A4F-A138-C6EDFF05F4AB}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{D0364854-C5F2-6A4F-A138-C6EDFF05F4AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="285">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="286">
   <si>
     <t>Name</t>
   </si>
@@ -892,6 +892,9 @@
   </si>
   <si>
     <t>Data/Command (SIO)</t>
+  </si>
+  <si>
+    <t>LDR</t>
   </si>
 </sst>
 </file>
@@ -920,7 +923,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="17">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1011,6 +1014,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -1098,9 +1107,6 @@
     <xf numFmtId="0" fontId="2" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -1148,6 +1154,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1722,7 +1731,7 @@
       <c r="B12" s="10">
         <v>10</v>
       </c>
-      <c r="C12" s="30" t="s">
+      <c r="C12" s="29" t="s">
         <v>11</v>
       </c>
       <c r="D12" s="5" t="s">
@@ -1741,7 +1750,7 @@
       <c r="B13" s="10">
         <v>11</v>
       </c>
-      <c r="C13" s="33" t="s">
+      <c r="C13" s="32" t="s">
         <v>12</v>
       </c>
       <c r="D13" s="5" t="s">
@@ -1760,7 +1769,7 @@
       <c r="B14" s="10">
         <v>12</v>
       </c>
-      <c r="C14" s="27" t="s">
+      <c r="C14" s="26" t="s">
         <v>13</v>
       </c>
       <c r="D14" s="5" t="s">
@@ -1781,7 +1790,7 @@
       <c r="B15" s="10">
         <v>13</v>
       </c>
-      <c r="C15" s="21" t="s">
+      <c r="C15" s="20" t="s">
         <v>14</v>
       </c>
       <c r="D15" s="5" t="s">
@@ -1821,7 +1830,7 @@
       <c r="B17" s="10">
         <v>15</v>
       </c>
-      <c r="C17" s="33" t="s">
+      <c r="C17" s="32" t="s">
         <v>16</v>
       </c>
       <c r="D17" s="5" t="s">
@@ -1926,7 +1935,7 @@
       <c r="B22" s="10">
         <v>20</v>
       </c>
-      <c r="C22" s="19" t="s">
+      <c r="C22" s="18" t="s">
         <v>21</v>
       </c>
       <c r="D22" s="5" t="s">
@@ -1968,7 +1977,7 @@
       <c r="B24" s="10">
         <v>22</v>
       </c>
-      <c r="C24" s="23" t="s">
+      <c r="C24" s="22" t="s">
         <v>97</v>
       </c>
       <c r="D24" s="5"/>
@@ -1985,7 +1994,7 @@
       <c r="B25" s="10">
         <v>23</v>
       </c>
-      <c r="C25" s="23" t="s">
+      <c r="C25" s="22" t="s">
         <v>98</v>
       </c>
       <c r="D25" s="5"/>
@@ -2002,10 +2011,10 @@
       <c r="B26" s="10">
         <v>24</v>
       </c>
-      <c r="C26" s="26" t="s">
+      <c r="C26" s="25" t="s">
         <v>99</v>
       </c>
-      <c r="D26" s="26" t="s">
+      <c r="D26" s="25" t="s">
         <v>101</v>
       </c>
       <c r="E26" s="5"/>
@@ -2021,10 +2030,10 @@
       <c r="B27" s="10">
         <v>25</v>
       </c>
-      <c r="C27" s="26" t="s">
+      <c r="C27" s="25" t="s">
         <v>100</v>
       </c>
-      <c r="D27" s="26" t="s">
+      <c r="D27" s="25" t="s">
         <v>102</v>
       </c>
       <c r="E27" s="5"/>
@@ -2103,16 +2112,16 @@
       <c r="A2" s="14">
         <v>0</v>
       </c>
-      <c r="B2" s="24" t="s">
+      <c r="B2" s="23" t="s">
         <v>98</v>
       </c>
-      <c r="C2" s="24" t="s">
+      <c r="C2" s="23" t="s">
         <v>94</v>
       </c>
       <c r="D2" s="13" t="s">
         <v>108</v>
       </c>
-      <c r="E2" s="24" t="s">
+      <c r="E2" s="23" t="s">
         <v>94</v>
       </c>
       <c r="F2" s="13" t="s">
@@ -2153,16 +2162,16 @@
       <c r="A3" s="14">
         <v>1</v>
       </c>
-      <c r="B3" s="24" t="s">
+      <c r="B3" s="23" t="s">
         <v>97</v>
       </c>
-      <c r="C3" s="24" t="s">
+      <c r="C3" s="23" t="s">
         <v>95</v>
       </c>
       <c r="D3" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="E3" s="24" t="s">
+      <c r="E3" s="23" t="s">
         <v>95</v>
       </c>
       <c r="F3" s="13" t="s">
@@ -2203,10 +2212,10 @@
       <c r="A4" s="14">
         <v>2</v>
       </c>
-      <c r="B4" s="18" t="s">
+      <c r="B4" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="17" t="s">
         <v>67</v>
       </c>
       <c r="D4" s="13" t="s">
@@ -2218,7 +2227,7 @@
       <c r="F4" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="G4" s="18" t="s">
+      <c r="G4" s="17" t="s">
         <v>67</v>
       </c>
       <c r="H4" s="13" t="s">
@@ -2253,10 +2262,10 @@
       <c r="A5" s="14">
         <v>3</v>
       </c>
-      <c r="B5" s="18" t="s">
+      <c r="B5" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="17" t="s">
         <v>68</v>
       </c>
       <c r="D5" s="13" t="s">
@@ -2268,7 +2277,7 @@
       <c r="F5" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="G5" s="18" t="s">
+      <c r="G5" s="17" t="s">
         <v>68</v>
       </c>
       <c r="H5" s="13" t="s">
@@ -2303,10 +2312,10 @@
       <c r="A6" s="14">
         <v>4</v>
       </c>
-      <c r="B6" s="18" t="s">
+      <c r="B6" s="17" t="s">
         <v>5</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="17" t="s">
         <v>69</v>
       </c>
       <c r="D6" s="13" t="s">
@@ -2318,7 +2327,7 @@
       <c r="F6" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="G6" s="18" t="s">
+      <c r="G6" s="17" t="s">
         <v>69</v>
       </c>
       <c r="H6" s="13" t="s">
@@ -2353,10 +2362,10 @@
       <c r="A7" s="14">
         <v>5</v>
       </c>
-      <c r="B7" s="18" t="s">
+      <c r="B7" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="17" t="s">
         <v>70</v>
       </c>
       <c r="D7" s="13" t="s">
@@ -2368,7 +2377,7 @@
       <c r="F7" s="13" t="s">
         <v>91</v>
       </c>
-      <c r="G7" s="18" t="s">
+      <c r="G7" s="17" t="s">
         <v>70</v>
       </c>
       <c r="H7" s="13" t="s">
@@ -2403,10 +2412,10 @@
       <c r="A8" s="14">
         <v>6</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="B8" s="17" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="17" t="s">
         <v>139</v>
       </c>
       <c r="D8" s="13" t="s">
@@ -2418,10 +2427,10 @@
       <c r="F8" s="13" t="s">
         <v>120</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="G8" s="17" t="s">
         <v>139</v>
       </c>
-      <c r="H8" s="17" t="s">
+      <c r="H8" s="13" t="s">
         <v>109</v>
       </c>
       <c r="I8" s="13" t="s">
@@ -2453,10 +2462,10 @@
       <c r="A9" s="14">
         <v>7</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="17" t="s">
         <v>144</v>
       </c>
       <c r="D9" s="13" t="s">
@@ -2468,7 +2477,7 @@
       <c r="F9" s="13" t="s">
         <v>126</v>
       </c>
-      <c r="G9" s="18" t="s">
+      <c r="G9" s="17" t="s">
         <v>144</v>
       </c>
       <c r="H9" s="13" t="s">
@@ -2503,22 +2512,22 @@
       <c r="A10" s="14">
         <v>8</v>
       </c>
-      <c r="B10" s="25" t="s">
+      <c r="B10" s="24" t="s">
         <v>99</v>
       </c>
-      <c r="C10" s="25" t="s">
+      <c r="C10" s="24" t="s">
         <v>103</v>
       </c>
       <c r="D10" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="E10" s="25" t="s">
+      <c r="E10" s="24" t="s">
         <v>103</v>
       </c>
       <c r="F10" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="G10" s="17" t="s">
+      <c r="G10" s="13" t="s">
         <v>149</v>
       </c>
       <c r="H10" s="13" t="s">
@@ -2553,16 +2562,16 @@
       <c r="A11" s="14">
         <v>9</v>
       </c>
-      <c r="B11" s="25" t="s">
+      <c r="B11" s="24" t="s">
         <v>100</v>
       </c>
-      <c r="C11" s="25" t="s">
+      <c r="C11" s="24" t="s">
         <v>104</v>
       </c>
       <c r="D11" s="13" t="s">
         <v>153</v>
       </c>
-      <c r="E11" s="25" t="s">
+      <c r="E11" s="24" t="s">
         <v>104</v>
       </c>
       <c r="F11" s="13" t="s">
@@ -2603,10 +2612,10 @@
       <c r="A12" s="14">
         <v>10</v>
       </c>
-      <c r="B12" s="32" t="s">
+      <c r="B12" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="32" t="s">
+      <c r="C12" s="31" t="s">
         <v>109</v>
       </c>
       <c r="D12" s="13" t="s">
@@ -2621,7 +2630,7 @@
       <c r="G12" s="13" t="s">
         <v>158</v>
       </c>
-      <c r="H12" s="32" t="s">
+      <c r="H12" s="31" t="s">
         <v>109</v>
       </c>
       <c r="I12" s="13" t="s">
@@ -2653,10 +2662,10 @@
       <c r="A13" s="14">
         <v>11</v>
       </c>
-      <c r="B13" s="32" t="s">
+      <c r="B13" s="31" t="s">
         <v>16</v>
       </c>
-      <c r="C13" s="32" t="s">
+      <c r="C13" s="31" t="s">
         <v>109</v>
       </c>
       <c r="D13" s="13" t="s">
@@ -2671,7 +2680,7 @@
       <c r="G13" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="H13" s="32" t="s">
+      <c r="H13" s="31" t="s">
         <v>109</v>
       </c>
       <c r="I13" s="13" t="s">
@@ -2703,10 +2712,10 @@
       <c r="A14" s="14">
         <v>12</v>
       </c>
-      <c r="B14" s="22" t="s">
+      <c r="B14" s="21" t="s">
         <v>15</v>
       </c>
-      <c r="C14" s="22" t="s">
+      <c r="C14" s="21" t="s">
         <v>90</v>
       </c>
       <c r="D14" s="13" t="s">
@@ -2715,7 +2724,7 @@
       <c r="E14" s="13" t="s">
         <v>94</v>
       </c>
-      <c r="F14" s="22" t="s">
+      <c r="F14" s="21" t="s">
         <v>90</v>
       </c>
       <c r="G14" s="13" t="s">
@@ -2753,10 +2762,10 @@
       <c r="A15" s="14">
         <v>13</v>
       </c>
-      <c r="B15" s="22" t="s">
+      <c r="B15" s="21" t="s">
         <v>14</v>
       </c>
-      <c r="C15" s="22" t="s">
+      <c r="C15" s="21" t="s">
         <v>91</v>
       </c>
       <c r="D15" s="13" t="s">
@@ -2765,7 +2774,7 @@
       <c r="E15" s="13" t="s">
         <v>95</v>
       </c>
-      <c r="F15" s="22" t="s">
+      <c r="F15" s="21" t="s">
         <v>91</v>
       </c>
       <c r="G15" s="13" t="s">
@@ -2803,10 +2812,10 @@
       <c r="A16" s="14">
         <v>14</v>
       </c>
-      <c r="B16" s="29" t="s">
+      <c r="B16" s="28" t="s">
         <v>3</v>
       </c>
-      <c r="C16" s="29" t="s">
+      <c r="C16" s="28" t="s">
         <v>109</v>
       </c>
       <c r="D16" s="13" t="s">
@@ -2821,7 +2830,7 @@
       <c r="G16" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="H16" s="29" t="s">
+      <c r="H16" s="28" t="s">
         <v>109</v>
       </c>
       <c r="I16" s="13" t="s">
@@ -2853,10 +2862,10 @@
       <c r="A17" s="14">
         <v>15</v>
       </c>
-      <c r="B17" s="20" t="s">
+      <c r="B17" s="19" t="s">
         <v>44</v>
       </c>
-      <c r="C17" s="20" t="s">
+      <c r="C17" s="19" t="s">
         <v>109</v>
       </c>
       <c r="D17" s="13" t="s">
@@ -2871,7 +2880,7 @@
       <c r="G17" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="H17" s="20" t="s">
+      <c r="H17" s="19" t="s">
         <v>109</v>
       </c>
       <c r="I17" s="13" t="s">
@@ -2899,14 +2908,14 @@
         <v>261</v>
       </c>
     </row>
-    <row r="18" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A18" s="14">
         <v>16</v>
       </c>
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="20" t="s">
+      <c r="C18" s="19" t="s">
         <v>65</v>
       </c>
       <c r="D18" s="13" t="s">
@@ -2918,7 +2927,7 @@
       <c r="F18" s="13" t="s">
         <v>90</v>
       </c>
-      <c r="G18" s="20" t="s">
+      <c r="G18" s="19" t="s">
         <v>65</v>
       </c>
       <c r="H18" s="13" t="s">
@@ -2953,13 +2962,13 @@
       <c r="A19" s="14">
         <v>17</v>
       </c>
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="19" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="20" t="s">
+      <c r="C19" s="19" t="s">
         <v>268</v>
       </c>
-      <c r="D19" s="20" t="s">
+      <c r="D19" s="19" t="s">
         <v>114</v>
       </c>
       <c r="E19" s="13" t="s">
@@ -2971,7 +2980,7 @@
       <c r="G19" s="13" t="s">
         <v>66</v>
       </c>
-      <c r="H19" s="20" t="s">
+      <c r="H19" s="19" t="s">
         <v>109</v>
       </c>
       <c r="I19" s="13" t="s">
@@ -3003,13 +3012,13 @@
       <c r="A20" s="14">
         <v>18</v>
       </c>
-      <c r="B20" s="20" t="s">
+      <c r="B20" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="C20" s="20" t="s">
+      <c r="C20" s="19" t="s">
         <v>78</v>
       </c>
-      <c r="D20" s="20" t="s">
+      <c r="D20" s="19" t="s">
         <v>78</v>
       </c>
       <c r="E20" s="13" t="s">
@@ -3053,13 +3062,13 @@
       <c r="A21" s="14">
         <v>19</v>
       </c>
-      <c r="B21" s="20" t="s">
+      <c r="B21" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="C21" s="20" t="s">
+      <c r="C21" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="D21" s="20" t="s">
+      <c r="D21" s="19" t="s">
         <v>124</v>
       </c>
       <c r="E21" s="13" t="s">
@@ -3103,10 +3112,10 @@
       <c r="A22" s="14">
         <v>20</v>
       </c>
-      <c r="B22" s="20" t="s">
+      <c r="B22" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="C22" s="20" t="s">
+      <c r="C22" s="19" t="s">
         <v>109</v>
       </c>
       <c r="D22" s="13" t="s">
@@ -3121,7 +3130,7 @@
       <c r="G22" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="H22" s="20" t="s">
+      <c r="H22" s="19" t="s">
         <v>109</v>
       </c>
       <c r="I22" s="13" t="s">
@@ -3293,7 +3302,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="26" spans="1:16" ht="27.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A26" s="15">
         <v>24</v>
       </c>
@@ -3441,10 +3450,10 @@
       <c r="A29" s="14">
         <v>27</v>
       </c>
-      <c r="B29" s="28" t="s">
+      <c r="B29" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="C29" s="28" t="s">
+      <c r="C29" s="27" t="s">
         <v>109</v>
       </c>
       <c r="D29" s="13" t="s">
@@ -3459,7 +3468,7 @@
       <c r="G29" s="13" t="s">
         <v>162</v>
       </c>
-      <c r="H29" s="28" t="s">
+      <c r="H29" s="27" t="s">
         <v>109</v>
       </c>
       <c r="I29" s="13" t="s">
@@ -3491,13 +3500,13 @@
       <c r="A30" s="14">
         <v>28</v>
       </c>
-      <c r="B30" s="31" t="s">
+      <c r="B30" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="C30" s="31" t="s">
+      <c r="C30" s="30" t="s">
         <v>148</v>
       </c>
-      <c r="D30" s="31" t="s">
+      <c r="D30" s="30" t="s">
         <v>148</v>
       </c>
       <c r="E30" s="13" t="s">
@@ -3541,13 +3550,13 @@
       <c r="A31" s="14">
         <v>29</v>
       </c>
-      <c r="B31" s="31" t="s">
+      <c r="B31" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="C31" s="31" t="s">
+      <c r="C31" s="30" t="s">
         <v>269</v>
       </c>
-      <c r="D31" s="31" t="s">
+      <c r="D31" s="30" t="s">
         <v>153</v>
       </c>
       <c r="E31" s="13" t="s">
@@ -3559,7 +3568,7 @@
       <c r="G31" s="13" t="s">
         <v>170</v>
       </c>
-      <c r="H31" s="31" t="s">
+      <c r="H31" s="30" t="s">
         <v>109</v>
       </c>
       <c r="I31" s="13" t="s">
@@ -3591,13 +3600,13 @@
       <c r="A32" s="14">
         <v>30</v>
       </c>
-      <c r="B32" s="31" t="s">
+      <c r="B32" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C32" s="31" t="s">
+      <c r="C32" s="30" t="s">
         <v>107</v>
       </c>
-      <c r="D32" s="31" t="s">
+      <c r="D32" s="30" t="s">
         <v>107</v>
       </c>
       <c r="E32" s="13" t="s">
@@ -3641,11 +3650,11 @@
       <c r="A33" s="14">
         <v>31</v>
       </c>
-      <c r="B33" s="13" t="s">
-        <v>265</v>
-      </c>
-      <c r="C33" s="13" t="s">
-        <v>59</v>
+      <c r="B33" s="33" t="s">
+        <v>285</v>
+      </c>
+      <c r="C33" s="33" t="s">
+        <v>242</v>
       </c>
       <c r="D33" s="13" t="s">
         <v>81</v>
@@ -3677,7 +3686,7 @@
       <c r="M33" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="N33" s="13" t="s">
+      <c r="N33" s="33" t="s">
         <v>242</v>
       </c>
       <c r="O33" s="13" t="s">

</xml_diff>

<commit_message>
fixed things for ldr pin
</commit_message>
<xml_diff>
--- a/ProjectPinAssignments.xlsx
+++ b/ProjectPinAssignments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ECE264\362_smart_knob\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22CC351A-8DAB-49D0-9EBC-DFE290766685}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7FF774F-471E-4339-9B66-F996044052A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{D0364854-C5F2-6A4F-A138-C6EDFF05F4AB}"/>
   </bookViews>
@@ -1063,7 +1063,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1156,6 +1156,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3437,7 +3440,7 @@
         <v>59</v>
       </c>
       <c r="N28" s="16" t="s">
-        <v>237</v>
+        <v>59</v>
       </c>
       <c r="O28" s="16" t="s">
         <v>59</v>
@@ -3487,7 +3490,7 @@
         <v>59</v>
       </c>
       <c r="N29" s="13" t="s">
-        <v>238</v>
+        <v>59</v>
       </c>
       <c r="O29" s="13" t="s">
         <v>59</v>
@@ -3537,7 +3540,7 @@
         <v>133</v>
       </c>
       <c r="N30" s="13" t="s">
-        <v>239</v>
+        <v>59</v>
       </c>
       <c r="O30" s="13" t="s">
         <v>262</v>
@@ -3587,7 +3590,7 @@
         <v>137</v>
       </c>
       <c r="N31" s="13" t="s">
-        <v>240</v>
+        <v>59</v>
       </c>
       <c r="O31" s="13" t="s">
         <v>262</v>
@@ -3637,7 +3640,7 @@
         <v>59</v>
       </c>
       <c r="N32" s="13" t="s">
-        <v>241</v>
+        <v>59</v>
       </c>
       <c r="O32" s="13" t="s">
         <v>262</v>
@@ -3650,11 +3653,11 @@
       <c r="A33" s="14">
         <v>31</v>
       </c>
-      <c r="B33" s="33" t="s">
-        <v>285</v>
-      </c>
-      <c r="C33" s="33" t="s">
-        <v>242</v>
+      <c r="B33" s="13" t="s">
+        <v>265</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>59</v>
       </c>
       <c r="D33" s="13" t="s">
         <v>81</v>
@@ -3686,8 +3689,8 @@
       <c r="M33" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="N33" s="33" t="s">
-        <v>242</v>
+      <c r="N33" s="34" t="s">
+        <v>59</v>
       </c>
       <c r="O33" s="13" t="s">
         <v>262</v>
@@ -4100,11 +4103,11 @@
       <c r="A42" s="14">
         <v>40</v>
       </c>
-      <c r="B42" s="13" t="s">
-        <v>265</v>
-      </c>
-      <c r="C42" s="13" t="s">
-        <v>59</v>
+      <c r="B42" s="33" t="s">
+        <v>285</v>
+      </c>
+      <c r="C42" s="33" t="s">
+        <v>242</v>
       </c>
       <c r="D42" s="13" t="s">
         <v>148</v>
@@ -4136,7 +4139,7 @@
       <c r="M42" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="N42" s="13" t="s">
+      <c r="N42" s="33" t="s">
         <v>237</v>
       </c>
       <c r="O42" s="13" t="s">

</xml_diff>

<commit_message>
started with motor control stuff
</commit_message>
<xml_diff>
--- a/ProjectPinAssignments.xlsx
+++ b/ProjectPinAssignments.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ECE264\362_smart_knob\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tyfor\OneDrive\Desktop\ECE362\362_smart_knob\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7FF774F-471E-4339-9B66-F996044052A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6504979B-DC91-401B-8AA4-201E04D2FE1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="9960" activeTab="1" xr2:uid="{D0364854-C5F2-6A4F-A138-C6EDFF05F4AB}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{D0364854-C5F2-6A4F-A138-C6EDFF05F4AB}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -21,23 +21,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="852" uniqueCount="287">
   <si>
     <t>Name</t>
   </si>
@@ -895,6 +884,9 @@
   </si>
   <si>
     <t>LDR</t>
+  </si>
+  <si>
+    <t>TMC_VIO</t>
   </si>
 </sst>
 </file>
@@ -1063,7 +1055,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1158,9 +1150,6 @@
     <xf numFmtId="0" fontId="2" fillId="16" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1169,6 +1158,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFBE2D5"/>
       <color rgb="FFC1F0C8"/>
       <color rgb="FFCAEDFB"/>
       <color rgb="FF66FFCC"/>
@@ -1176,7 +1166,6 @@
       <color rgb="FFFFFF99"/>
       <color rgb="FF9999FF"/>
       <color rgb="FFF2CEEF"/>
-      <color rgb="FFFBE2D5"/>
       <color rgb="FFDE7272"/>
     </mruColors>
   </colors>
@@ -3689,7 +3678,7 @@
       <c r="M33" s="13" t="s">
         <v>59</v>
       </c>
-      <c r="N33" s="34" t="s">
+      <c r="N33" s="13" t="s">
         <v>59</v>
       </c>
       <c r="O33" s="13" t="s">
@@ -4153,11 +4142,11 @@
       <c r="A43" s="14">
         <v>41</v>
       </c>
-      <c r="B43" s="13" t="s">
-        <v>265</v>
-      </c>
-      <c r="C43" s="13" t="s">
-        <v>59</v>
+      <c r="B43" s="17" t="s">
+        <v>286</v>
+      </c>
+      <c r="C43" s="17" t="s">
+        <v>109</v>
       </c>
       <c r="D43" s="13" t="s">
         <v>153</v>
@@ -4171,7 +4160,7 @@
       <c r="G43" s="13" t="s">
         <v>230</v>
       </c>
-      <c r="H43" s="13" t="s">
+      <c r="H43" s="17" t="s">
         <v>109</v>
       </c>
       <c r="I43" s="13" t="s">

</xml_diff>